<commit_message>
Some architectures have been modified and an AI self-healing function has been added. When the steps fail to proceed, the RAG AI will be triggered. It will attempt to continue the steps based on the understanding of the known requirements.
</commit_message>
<xml_diff>
--- a/use_cases/2025 DEC 1225 Smoke testing on prod env.xlsx
+++ b/use_cases/2025 DEC 1225 Smoke testing on prod env.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="72">
   <si>
     <t>ID</t>
   </si>
@@ -317,6 +317,42 @@
 3. 3. Checkbox is checked and selection is registered.
 4. 4. Selected poster is added to the ticket product media section.</t>
   </si>
+  <si>
+    <t>T4777</t>
+  </si>
+  <si>
+    <t>Verify when "Enable co-selling by default" is on, create an event post, the resale setting will be turned on</t>
+  </si>
+  <si>
+    <r>
+      <t>1. turn on "Enable co-selling by default" and set the default commission rate
+2. create an event post from: 
+event list,
+event landing page&gt;more action,
+event landing page&gt;Event&gt;Posts&gt;Create a post,
++button&gt;Create a post</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="宋体"/>
+        <charset val="0"/>
+      </rPr>
+      <t>，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Verdana"/>
+        <charset val="0"/>
+      </rPr>
+      <t xml:space="preserve">
+post module&gt;Add new</t>
+    </r>
+  </si>
+  <si>
+    <t>the resale setting will be turned on and it will use the ticket and merch commission rate</t>
+  </si>
 </sst>
 </file>
 
@@ -328,7 +364,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="12"/>
       <name val="Verdana"/>
@@ -484,6 +520,11 @@
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="宋体"/>
+      <charset val="0"/>
     </font>
   </fonts>
   <fills count="33">
@@ -803,7 +844,7 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1555,7 +1596,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="12" width="11" style="1" customWidth="1"/>
@@ -1901,6 +1942,35 @@
       </c>
       <c r="L9" s="1" t="s">
         <v>67</v>
+      </c>
+    </row>
+    <row r="10" ht="306" customHeight="1" spans="1:12">
+      <c r="A10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>